<commit_message>
Removing image from BillboardMasterSeeder
</commit_message>
<xml_diff>
--- a/public/UbicacionesVallasV2.xlsx
+++ b/public/UbicacionesVallasV2.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3209" uniqueCount="1099">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3222" uniqueCount="1106">
   <si>
     <t xml:space="preserve">TIPO DE ESTRUCTURA</t>
   </si>
@@ -3320,6 +3320,27 @@
   </si>
   <si>
     <t xml:space="preserve">-16.5250278,-68.1482222</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIGITAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100-A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frente a la Corte de Justicia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cara mira hacia Av. 6  de agosto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6X3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maps.app.goo.gl/bMv5qfn8qt6rVf4y9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-14.835596, -64.903506</t>
   </si>
 </sst>
 </file>
@@ -3650,7 +3671,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="31.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="1" width="11.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="30.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="25.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="33.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="11.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="21.9"/>
@@ -17483,23 +17504,51 @@
       <c r="Z246" s="3"/>
     </row>
     <row r="247" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A247" s="3"/>
-      <c r="B247" s="3"/>
-      <c r="C247" s="3"/>
-      <c r="D247" s="3"/>
-      <c r="E247" s="3"/>
-      <c r="F247" s="3"/>
-      <c r="G247" s="3"/>
-      <c r="H247" s="3"/>
-      <c r="I247" s="3"/>
-      <c r="J247" s="3"/>
-      <c r="K247" s="3"/>
-      <c r="L247" s="3"/>
-      <c r="M247" s="3"/>
-      <c r="N247" s="3"/>
-      <c r="O247" s="3"/>
-      <c r="P247" s="3"/>
-      <c r="Q247" s="3"/>
+      <c r="A247" s="16" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B247" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="C247" s="5" t="s">
+        <v>974</v>
+      </c>
+      <c r="D247" s="16" t="s">
+        <v>975</v>
+      </c>
+      <c r="E247" s="4" t="s">
+        <v>1100</v>
+      </c>
+      <c r="F247" s="14" t="s">
+        <v>1101</v>
+      </c>
+      <c r="G247" s="5" t="s">
+        <v>1102</v>
+      </c>
+      <c r="H247" s="14"/>
+      <c r="I247" s="16" t="s">
+        <v>1103</v>
+      </c>
+      <c r="J247" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="K247" s="17" t="n">
+        <v>6200</v>
+      </c>
+      <c r="L247" s="6" t="s">
+        <v>1104</v>
+      </c>
+      <c r="M247" s="6" t="s">
+        <v>1105</v>
+      </c>
+      <c r="N247" s="5"/>
+      <c r="O247" s="15"/>
+      <c r="P247" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q247" s="9" t="s">
+        <v>416</v>
+      </c>
       <c r="R247" s="3"/>
       <c r="S247" s="3"/>
       <c r="T247" s="3"/>

</xml_diff>

<commit_message>
Added new field to organizations
</commit_message>
<xml_diff>
--- a/public/UbicacionesVallasV2.xlsx
+++ b/public/UbicacionesVallasV2.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sheet3" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet3!$A$1:$Q$246</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet3!$A$1:$Q$247</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -38720,7 +38720,7 @@
       <c r="Z1000" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q246"/>
+  <autoFilter ref="A1:Q247"/>
   <hyperlinks>
     <hyperlink ref="L3" r:id="rId1" display="https://maps.app.goo.gl/eg1cMcUP1zrxFe6h9"/>
     <hyperlink ref="L37" r:id="rId2" display="https://maps.app.goo.gl/QUgqpH1fcNoEYXdq5"/>

</xml_diff>